<commit_message>
feat: taggear numero da venda para pedidos multilinhas e evitar repeticao
</commit_message>
<xml_diff>
--- a/exemplos/exemplo_vendas_upseller.xlsx
+++ b/exemplos/exemplo_vendas_upseller.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>Preço de Produto</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Número da Venda</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -477,6 +482,7 @@
           <t>R$ 85,00</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -507,6 +513,7 @@
           <t>R$ 89,90</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -537,13 +544,10 @@
           <t>R$ 119,90</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>241006J1K2L3</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>VAR_SHN_301</t>
@@ -565,6 +569,73 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>R$ 55,00</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>241006J1K2L3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VAR_SHP_101</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>POLO-AZUL-M</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Camisa Polo Algodão Pima Confort</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>R$ 85,00</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>241006MULTI_99</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VAR_SHP_102</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>POLO-PRETA-G</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Camisa Polo Algodão Pima Confort</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>R$ 89,90</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>241006MULTI_99</t>
         </is>
       </c>
     </row>

</xml_diff>